<commit_message>
GR12 run with hard period spreading: 207→202 conflicts, 87.1% placement
Period spreading now HARD constraint — sections must use unique periods
before doubling up. Key improvements:
- 642 PE: 11→3 conflicts (-8)
- 742 Economics: 15→12 (-3)
- 543 Anatomy H: 9→6 (-3)
- 955 Academic Support: 7→4 (-3)
- 763 AP Gov: 6→3 (-3)
- AP/Honors fulfillment: 92.6%→96.3%

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/Job1_Section_Placements_GR12_2026_27.xlsx
+++ b/Job1_Section_Placements_GR12_2026_27.xlsx
@@ -6403,7 +6403,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J80" s="2" t="inlineStr">
@@ -6477,7 +6477,7 @@
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J81" s="2" t="inlineStr">
@@ -6551,7 +6551,7 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
@@ -6847,7 +6847,7 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J86" s="2" t="inlineStr">
@@ -6921,7 +6921,7 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J87" s="2" t="inlineStr">
@@ -6995,7 +6995,7 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J88" s="2" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J91" s="2" t="inlineStr">
@@ -7587,7 +7587,7 @@
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
@@ -7661,7 +7661,7 @@
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
@@ -7809,7 +7809,7 @@
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J99" s="2" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="I100" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J100" s="2" t="inlineStr">
@@ -7957,7 +7957,7 @@
       </c>
       <c r="I101" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J101" s="2" t="inlineStr">
@@ -8031,7 +8031,7 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J102" s="2" t="inlineStr">
@@ -8105,7 +8105,7 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J103" s="2" t="inlineStr">
@@ -8179,7 +8179,7 @@
       </c>
       <c r="I104" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J104" s="2" t="inlineStr">
@@ -8327,7 +8327,7 @@
       </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J106" s="2" t="inlineStr">
@@ -8401,7 +8401,7 @@
       </c>
       <c r="I107" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J107" s="2" t="inlineStr">
@@ -8549,7 +8549,7 @@
       </c>
       <c r="I109" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J109" s="2" t="inlineStr">
@@ -8623,7 +8623,7 @@
       </c>
       <c r="I110" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J110" s="2" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="I111" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J111" s="2" t="inlineStr">
@@ -8771,7 +8771,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="I113" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J113" s="2" t="inlineStr">
@@ -8919,7 +8919,7 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="I115" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J115" s="2" t="inlineStr">
@@ -9067,7 +9067,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -9141,7 +9141,7 @@
       </c>
       <c r="I117" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
@@ -9215,7 +9215,7 @@
       </c>
       <c r="I118" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J118" s="2" t="inlineStr">
@@ -9289,7 +9289,7 @@
       </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J119" s="2" t="inlineStr">
@@ -9363,7 +9363,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -9437,7 +9437,7 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
@@ -9659,7 +9659,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -9881,7 +9881,7 @@
       </c>
       <c r="I127" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J127" s="2" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="I128" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J128" s="2" t="inlineStr">
@@ -10103,7 +10103,7 @@
       </c>
       <c r="I130" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J130" s="2" t="inlineStr">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -10251,7 +10251,7 @@
       </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J132" s="2" t="inlineStr">
@@ -10399,7 +10399,7 @@
       </c>
       <c r="I134" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J134" s="2" t="inlineStr">
@@ -10547,7 +10547,7 @@
       </c>
       <c r="I136" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J136" s="2" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="I137" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J137" s="2" t="inlineStr">
@@ -10695,7 +10695,7 @@
       </c>
       <c r="I138" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J138" s="2" t="inlineStr">
@@ -10769,7 +10769,7 @@
       </c>
       <c r="I139" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J139" s="2" t="inlineStr">
@@ -10843,7 +10843,7 @@
       </c>
       <c r="I140" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J140" s="2" t="inlineStr">
@@ -10917,7 +10917,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="I142" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J142" s="2" t="inlineStr">
@@ -11065,7 +11065,7 @@
       </c>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr">
@@ -11139,7 +11139,7 @@
       </c>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr">
@@ -11213,7 +11213,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -11287,7 +11287,7 @@
       </c>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>E</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="I147" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J147" s="2" t="inlineStr">
@@ -11435,7 +11435,7 @@
       </c>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr">
@@ -11583,7 +11583,7 @@
       </c>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>G</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr">
@@ -11657,7 +11657,7 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>F</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr">
@@ -11805,7 +11805,7 @@
       </c>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr">
@@ -12027,7 +12027,7 @@
       </c>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>D</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr">
@@ -12323,7 +12323,7 @@
       </c>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr">
@@ -13968,16 +13968,16 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3">
@@ -13987,16 +13987,16 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>18</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -14006,13 +14006,13 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" s="3" t="n">
         <v>26</v>
@@ -14028,13 +14028,13 @@
         <v>6</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -14044,16 +14044,16 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -14063,16 +14063,16 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -14082,16 +14082,16 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>6</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -16027,7 +16027,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>75/160</t>
+          <t>71/160</t>
         </is>
       </c>
     </row>
@@ -16050,7 +16050,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
@@ -16060,7 +16060,7 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -16080,7 +16080,7 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -16090,7 +16090,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16">
@@ -16100,7 +16100,7 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -16110,7 +16110,7 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>